<commit_message>
feat: implement group-based Written Capstone compliance tracking and consolidate Lema/Alvear project defense in schedule
</commit_message>
<xml_diff>
--- a/data/presentaciones_crcronograma.xlsx
+++ b/data/presentaciones_crcronograma.xlsx
@@ -10587,359 +10587,361 @@
         <v>1</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
-        <is>
-          <t>Detección de noticias falsas mediante técnicas de Inteligencia Artificial aplicadas al Procesamiento de Lenguaje Natural en el contexto periodístico</t>
-        </is>
-      </c>
-      <c r="I117" s="2" t="inlineStr">
-        <is>
-          <t>SABADO</t>
-        </is>
-      </c>
-      <c r="J117" s="2" t="n">
-        <v>226</v>
-      </c>
-      <c r="K117" s="2" t="inlineStr">
-        <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
-        </is>
-      </c>
-      <c r="L117" s="2" t="inlineStr">
-        <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
-        </is>
-      </c>
-      <c r="M117" s="2" t="inlineStr">
-        <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO</t>
-        </is>
-      </c>
-      <c r="N117" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="O117" s="2" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="P117" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="Q117" s="2" t="inlineStr">
-        <is>
-          <t>11:00 - 11:30</t>
-        </is>
-      </c>
-      <c r="R117" s="2" t="inlineStr">
-        <is>
-          <t>Sala 1</t>
-        </is>
-      </c>
-      <c r="S117" s="2" t="inlineStr">
-        <is>
-          <t>PATRICIO DAVID PONCE</t>
-        </is>
-      </c>
-      <c r="T117" s="2" t="n"/>
-    </row>
-    <row r="118" ht="60" customHeight="1">
-      <c r="A118" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B118" s="2" t="n">
-        <v>1718453259</v>
-      </c>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>A00026452</t>
-        </is>
-      </c>
-      <c r="D118" s="2" t="inlineStr">
-        <is>
-          <t>TALLANA FARINANGO LUIS GUILLERMO</t>
-        </is>
-      </c>
-      <c r="E118" s="2" t="inlineStr">
-        <is>
-          <t>luis.tallana@udla.edu.ec</t>
-        </is>
-      </c>
-      <c r="F118" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G118" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="H118" s="2" t="inlineStr">
-        <is>
-          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
-        </is>
-      </c>
-      <c r="I118" s="2" t="inlineStr">
-        <is>
-          <t>MIERCOLES</t>
-        </is>
-      </c>
-      <c r="J118" s="2" t="n">
-        <v>223</v>
-      </c>
-      <c r="K118" s="2" t="inlineStr">
-        <is>
-          <t>DAVID POZO ESPÍN</t>
-        </is>
-      </c>
-      <c r="L118" s="2" t="inlineStr">
-        <is>
-          <t>LEONARDO ARÉVALO RIVERA</t>
-        </is>
-      </c>
-      <c r="M118" s="2" t="inlineStr">
-        <is>
-          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
-        </is>
-      </c>
-      <c r="N118" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O118" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="P118" s="2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="Q118" s="2" t="inlineStr">
-        <is>
-          <t>11:30 - 12:00</t>
-        </is>
-      </c>
-      <c r="R118" s="2" t="inlineStr">
-        <is>
-          <t>Sala 2</t>
-        </is>
-      </c>
-      <c r="S118" s="2" t="inlineStr">
-        <is>
-          <t>MARCO GALARZA CASTILLO</t>
-        </is>
-      </c>
-      <c r="T118" s="2" t="n"/>
-    </row>
-    <row r="119" ht="45" customHeight="1">
-      <c r="A119" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B119" s="2" t="n">
-        <v>1714286448</v>
-      </c>
-      <c r="C119" s="2" t="inlineStr">
-        <is>
-          <t>A00875711</t>
-        </is>
-      </c>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>MENESES SAENZ HOMERO FRANCISCO</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
-          <t>homero.meneses.saenz@udla.edu.ec</t>
-        </is>
-      </c>
-      <c r="F119" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G119" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="H119" s="2" t="inlineStr">
-        <is>
-          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
-        </is>
-      </c>
-      <c r="I119" s="2" t="inlineStr">
-        <is>
-          <t>MIERCOLES</t>
-        </is>
-      </c>
-      <c r="J119" s="2" t="n">
-        <v>223</v>
-      </c>
-      <c r="K119" s="2" t="inlineStr">
-        <is>
-          <t>DAVID POZO ESPÍN</t>
-        </is>
-      </c>
-      <c r="L119" s="2" t="inlineStr">
-        <is>
-          <t>LEONARDO ARÉVALO RIVERA</t>
-        </is>
-      </c>
-      <c r="M119" s="2" t="inlineStr">
-        <is>
-          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
-        </is>
-      </c>
-      <c r="N119" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O119" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="P119" s="2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="Q119" s="2" t="inlineStr">
-        <is>
-          <t>11:30 - 12:00</t>
-        </is>
-      </c>
-      <c r="R119" s="2" t="inlineStr">
-        <is>
-          <t>Sala 2</t>
-        </is>
-      </c>
-      <c r="S119" s="2" t="inlineStr">
-        <is>
-          <t>MARCO GALARZA CASTILLO</t>
-        </is>
-      </c>
-      <c r="T119" s="2" t="n"/>
-    </row>
-    <row r="120" ht="45" customHeight="1">
-      <c r="A120" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B120" s="2" t="n">
-        <v>1721548756</v>
-      </c>
-      <c r="C120" s="2" t="inlineStr">
-        <is>
-          <t>A00135371</t>
-        </is>
-      </c>
-      <c r="D120" s="2" t="inlineStr">
-        <is>
-          <t>QUELAL CRUZ JONATHAN DAVID</t>
-        </is>
-      </c>
-      <c r="E120" s="2" t="inlineStr">
-        <is>
-          <t>jonathan.quelal@udla.edu.ec</t>
-        </is>
-      </c>
-      <c r="F120" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G120" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="H120" s="2" t="inlineStr">
-        <is>
-          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
-        </is>
-      </c>
-      <c r="I120" s="2" t="inlineStr">
-        <is>
-          <t>MIERCOLES</t>
-        </is>
-      </c>
-      <c r="J120" s="2" t="n">
-        <v>223</v>
-      </c>
-      <c r="K120" s="2" t="inlineStr">
-        <is>
-          <t>DAVID POZO ESPÍN</t>
-        </is>
-      </c>
-      <c r="L120" s="2" t="inlineStr">
-        <is>
-          <t>LEONARDO ARÉVALO RIVERA</t>
-        </is>
-      </c>
-      <c r="M120" s="2" t="inlineStr">
-        <is>
-          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
-        </is>
-      </c>
-      <c r="N120" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O120" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="P120" s="2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="Q120" s="2" t="inlineStr">
-        <is>
-          <t>11:30 - 12:00</t>
-        </is>
-      </c>
-      <c r="R120" s="2" t="inlineStr">
-        <is>
-          <t>Sala 2</t>
-        </is>
-      </c>
-      <c r="S120" s="2" t="inlineStr">
-        <is>
-          <t>MARCO GALARZA CASTILLO</t>
-        </is>
-      </c>
-      <c r="T120" s="2" t="n"/>
-    </row>
-    <row r="121" ht="45" customHeight="1">
-      <c r="A121" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B121" s="2" t="n">
-        <v>1716255763</v>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>A00018648</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>ALVEAR LEMA EMILIO JOSE</t>
-        </is>
-      </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>emilio.alvear@udla.edu.ec</t>
-        </is>
-      </c>
-      <c r="F121" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G121" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="H121" s="2" t="inlineStr">
         <is>
           <t>Sistema inteligente de automatización, predicción y atención asistida para 
 optimizar la gestión de casos en soporte técnico para la empresa 
 Hispasat en Ecuador</t>
         </is>
       </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>SABADO</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="n">
+        <v>226</v>
+      </c>
+      <c r="K117" s="2" t="inlineStr">
+        <is>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+        </is>
+      </c>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+        </is>
+      </c>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
+        </is>
+      </c>
+      <c r="N117" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="P117" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="Q117" s="2" t="inlineStr">
+        <is>
+          <t>11:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="R117" s="2" t="inlineStr">
+        <is>
+          <t>Sala 1</t>
+        </is>
+      </c>
+      <c r="S117" s="2" t="inlineStr">
+        <is>
+          <t>PATRICIO DAVID PONCE</t>
+        </is>
+      </c>
+      <c r="T117" s="2" t="n"/>
+    </row>
+    <row r="118" ht="60" customHeight="1">
+      <c r="A118" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B118" s="2" t="n">
+        <v>1718453259</v>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>A00026452</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>TALLANA FARINANGO LUIS GUILLERMO</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>luis.tallana@udla.edu.ec</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G118" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>MIERCOLES</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="n">
+        <v>223</v>
+      </c>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>DAVID POZO ESPÍN</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>LEONARDO ARÉVALO RIVERA</t>
+        </is>
+      </c>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
+        </is>
+      </c>
+      <c r="N118" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="P118" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="Q118" s="2" t="inlineStr">
+        <is>
+          <t>11:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="R118" s="2" t="inlineStr">
+        <is>
+          <t>Sala 2</t>
+        </is>
+      </c>
+      <c r="S118" s="2" t="inlineStr">
+        <is>
+          <t>MARCO GALARZA CASTILLO</t>
+        </is>
+      </c>
+      <c r="T118" s="2" t="n"/>
+    </row>
+    <row r="119" ht="45" customHeight="1">
+      <c r="A119" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B119" s="2" t="n">
+        <v>1714286448</v>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>A00875711</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>MENESES SAENZ HOMERO FRANCISCO</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>homero.meneses.saenz@udla.edu.ec</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G119" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>MIERCOLES</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="n">
+        <v>223</v>
+      </c>
+      <c r="K119" s="2" t="inlineStr">
+        <is>
+          <t>DAVID POZO ESPÍN</t>
+        </is>
+      </c>
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t>LEONARDO ARÉVALO RIVERA</t>
+        </is>
+      </c>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
+        </is>
+      </c>
+      <c r="N119" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O119" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="P119" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="Q119" s="2" t="inlineStr">
+        <is>
+          <t>11:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="R119" s="2" t="inlineStr">
+        <is>
+          <t>Sala 2</t>
+        </is>
+      </c>
+      <c r="S119" s="2" t="inlineStr">
+        <is>
+          <t>MARCO GALARZA CASTILLO</t>
+        </is>
+      </c>
+      <c r="T119" s="2" t="n"/>
+    </row>
+    <row r="120" ht="45" customHeight="1">
+      <c r="A120" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B120" s="2" t="n">
+        <v>1721548756</v>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>A00135371</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>QUELAL CRUZ JONATHAN DAVID</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>jonathan.quelal@udla.edu.ec</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G120" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>MIERCOLES</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="n">
+        <v>223</v>
+      </c>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>DAVID POZO ESPÍN</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>LEONARDO ARÉVALO RIVERA</t>
+        </is>
+      </c>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
+        </is>
+      </c>
+      <c r="N120" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O120" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="P120" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="Q120" s="2" t="inlineStr">
+        <is>
+          <t>11:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="R120" s="2" t="inlineStr">
+        <is>
+          <t>Sala 2</t>
+        </is>
+      </c>
+      <c r="S120" s="2" t="inlineStr">
+        <is>
+          <t>MARCO GALARZA CASTILLO</t>
+        </is>
+      </c>
+      <c r="T120" s="2" t="n"/>
+    </row>
+    <row r="121" ht="45" customHeight="1">
+      <c r="A121" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B121" s="2" t="n">
+        <v>1716255763</v>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>A00018648</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>ALVEAR LEMA EMILIO JOSE</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>emilio.alvear@udla.edu.ec</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G121" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>Sistema inteligente de automatización, predicción y atención asistida para 
+optimizar la gestión de casos en soporte técnico para la empresa 
+Hispasat en Ecuador</t>
+        </is>
+      </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
           <t>SABADO</t>
@@ -10960,7 +10962,7 @@
       </c>
       <c r="M121" s="2" t="inlineStr">
         <is>
-          <t>ALVEAR LEMA EMILIO JOSE</t>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
       <c r="N121" s="2" t="n">
@@ -17635,7 +17637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:M68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="14.1"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="2"/>
@@ -20921,65 +20923,65 @@
     </row>
     <row r="60" ht="45" customHeight="1">
       <c r="A60" s="2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B60" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>11:00 - 11:30</t>
+          <t>11:30 - 12:00</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Sala 1</t>
+          <t>Sala 2</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+          <t>DAVID POZO ESPÍN</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+          <t>LEONARDO ARÉVALO RIVERA</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>PATRICIO DAVID PONCE</t>
+          <t>MARCO GALARZA CASTILLO</t>
         </is>
       </c>
       <c r="H60" s="2" t="n"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Detección de noticias falsas mediante técnicas de Inteligencia Artificial aplicadas al Procesamiento de Lenguaje Natural en el contexto periodístico</t>
+          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO</t>
+          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
         </is>
       </c>
       <c r="K60" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>SABADO</t>
+          <t>MIERCOLES</t>
         </is>
       </c>
       <c r="M60" s="2" t="n">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="61" ht="45" customHeight="1">
       <c r="A61" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B61" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
@@ -20988,62 +20990,60 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Sala 2</t>
+          <t>Sala 1</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>DAVID POZO ESPÍN</t>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>LEONARDO ARÉVALO RIVERA</t>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>MARCO GALARZA CASTILLO</t>
+          <t>PATRICIO DAVID PONCE</t>
         </is>
       </c>
       <c r="H61" s="2" t="n"/>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
-        </is>
-      </c>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
-        </is>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>MIERCOLES</t>
+          <t>SABADO</t>
         </is>
       </c>
       <c r="M61" s="2" t="n">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="62" ht="45" customHeight="1">
       <c r="A62" s="2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B62" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>11:30 - 12:00</t>
+          <t>08:30 - 09:00</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Sala 1</t>
+          <t>Sala 2</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -21053,23 +21053,23 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+          <t>JUAN CARLOS FIGUEROA</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>PATRICIO DAVID PONCE</t>
+          <t>MARCO GALARZA CASTILLO</t>
         </is>
       </c>
       <c r="H62" s="2" t="n"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Sistema inteligente de automatización, predicción y atención asistida para  optimizar la gestión de casos en soporte técnico para la empresa  Hispasat en Ecuador</t>
+          <t>Sistema inteligente de captación, clasificación y predicción de oportunidades de venta mediante un agente de IA en WhatsApp para Clearminds Consultores.</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>ALVEAR LEMA EMILIO JOSE</t>
+          <t>VILLEGAS ALLAUCA ANTONIO DE JESUS</t>
         </is>
       </c>
       <c r="K62" s="2" t="n">
@@ -21077,7 +21077,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>SABADO</t>
+          <t>MIERCOLES</t>
         </is>
       </c>
       <c r="M62" s="2" t="n">
@@ -21086,124 +21086,124 @@
     </row>
     <row r="63" ht="45" customHeight="1">
       <c r="A63" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B63" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>08:30 - 09:00</t>
+          <t>09:30 - 10:00</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Sala 2</t>
+          <t>Sala 1</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>JUAN CARLOS FIGUEROA</t>
+          <t>ANDREA GALLEGOS ANDRADE</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>MARCO GALARZA CASTILLO</t>
+          <t>PATRICIO DAVID PONCE</t>
         </is>
       </c>
       <c r="H63" s="2" t="n"/>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Sistema inteligente de captación, clasificación y predicción de oportunidades de venta mediante un agente de IA en WhatsApp para Clearminds Consultores.</t>
+          <t>Análisis de sentimientos y clasificación de negocio para comentarios de encuestas de satisfacción de clientes.</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>VILLEGAS ALLAUCA ANTONIO DE JESUS</t>
+          <t>BEDON CAMPAÑA ADRIAN RUBEN / BEDON RODRIGUEZ JAIRO FABRISIO</t>
         </is>
       </c>
       <c r="K63" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>MIERCOLES</t>
+          <t>MARTES</t>
         </is>
       </c>
       <c r="M63" s="2" t="n">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="64" ht="45" customHeight="1">
       <c r="A64" s="2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>09:30 - 10:00</t>
+          <t>08:30 - 09:00</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Sala 1</t>
+          <t>Sala 2</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>ANDREA GALLEGOS ANDRADE</t>
+          <t>LUIS CRIOLLO</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>PATRICIO DAVID PONCE</t>
+          <t>MARCO GALARZA CASTILLO</t>
         </is>
       </c>
       <c r="H64" s="2" t="n"/>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Análisis de sentimientos y clasificación de negocio para comentarios de encuestas de satisfacción de clientes.</t>
+          <t>Predicción del riesgo de daño a uno mismo y a otros en consultantes que buscan  atención psicológica en un centro de formación en psicoterapia mediante  aprendizaje de máquina a partir de datos clínicos y sociodemográficos</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>BEDON CAMPAÑA ADRIAN RUBEN / BEDON RODRIGUEZ JAIRO FABRISIO</t>
+          <t>VALDIVIEZO OÑA JORGE ANDRES</t>
         </is>
       </c>
       <c r="K64" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>MARTES</t>
+          <t>SABADO</t>
         </is>
       </c>
       <c r="M64" s="2" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="2" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>08:30 - 09:00</t>
+          <t>09:30 - 10:00</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -21218,7 +21218,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>LUIS CRIOLLO</t>
+          <t>PABLO MONCAYO</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -21229,12 +21229,12 @@
       <c r="H65" s="2" t="n"/>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Predicción del riesgo de daño a uno mismo y a otros en consultantes que buscan  atención psicológica en un centro de formación en psicoterapia mediante  aprendizaje de máquina a partir de datos clínicos y sociodemográficos</t>
+          <t>Implementación de IA Generativa para los flujos de mercado entre  compañías para Nestlé S.A.</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>VALDIVIEZO OÑA JORGE ANDRES</t>
+          <t>POLO EGAS TAMIA EMILIA</t>
         </is>
       </c>
       <c r="K65" s="2" t="n">
@@ -21242,7 +21242,7 @@
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>SABADO</t>
+          <t>MIERCOLES</t>
         </is>
       </c>
       <c r="M65" s="2" t="n">
@@ -21251,124 +21251,124 @@
     </row>
     <row r="66" ht="60" customHeight="1">
       <c r="A66" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>09:30 - 10:00</t>
+          <t>12:00 - 12:30</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Sala 2</t>
+          <t>Sala 1</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>PABLO MONCAYO</t>
+          <t>MATEO FERNANDO CÓRDOVA PROAÑO</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>MARCO GALARZA CASTILLO</t>
+          <t>PATRICIO DAVID PONCE</t>
         </is>
       </c>
       <c r="H66" s="2" t="n"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Implementación de IA Generativa para los flujos de mercado entre  compañías para Nestlé S.A.</t>
+          <t>Implementación de un Proceso de Atención Digital mediante un Chatbot  con Inteligencia Artificial para la Mejora de la Atención al Usuario</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>POLO EGAS TAMIA EMILIA</t>
+          <t>ESPINOZA AGUILAR CAMILA ALEJANDRA / CUMBAL CUMBAL JOSE ALEXANDER</t>
         </is>
       </c>
       <c r="K66" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>MIERCOLES</t>
+          <t>MARTES</t>
         </is>
       </c>
       <c r="M66" s="2" t="n">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B67" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>12:00 - 12:30</t>
+          <t>09:30 - 10:00</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Sala 1</t>
+          <t>Sala 2</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>MATEO FERNANDO CÓRDOVA PROAÑO</t>
+          <t>IVÁN ORTIZ</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>PATRICIO DAVID PONCE</t>
+          <t>MARCO GALARZA CASTILLO</t>
         </is>
       </c>
       <c r="H67" s="2" t="n"/>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Implementación de un Proceso de Atención Digital mediante un Chatbot  con Inteligencia Artificial para la Mejora de la Atención al Usuario</t>
+          <t>Desarrollo de un agente inteligente basado en modelos de lenguaje de gran  escala para la automatización del análisis y respuesta a incidentes de  ciberseguridad</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>ESPINOZA AGUILAR CAMILA ALEJANDRA / CUMBAL CUMBAL JOSE ALEXANDER</t>
+          <t>BUITRON GONZAGA CRISTHIAN ANDRES</t>
         </is>
       </c>
       <c r="K67" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>MARTES</t>
+          <t>MIERCOLES</t>
         </is>
       </c>
       <c r="M67" s="2" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="68" ht="45" customHeight="1">
       <c r="A68" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B68" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>09:30 - 10:00</t>
+          <t>11:30 - 12:00</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -21383,7 +21383,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>IVÁN ORTIZ</t>
+          <t>JAIME FELIPE MEDINA SOTOMAYOR</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -21394,81 +21394,27 @@
       <c r="H68" s="2" t="n"/>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo de un agente inteligente basado en modelos de lenguaje de gran  escala para la automatización del análisis y respuesta a incidentes de  ciberseguridad</t>
+          <t>Modelo predictivo del rendimiento deportivo en el fútbol ecuatoriano a  partir del presupuesto institucional y variables competitivas usando  técnicas de Inteligencia Artificial</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>BUITRON GONZAGA CRISTHIAN ANDRES</t>
+          <t>CASTRO GARCIA DIEGO FERNANDO / PILA CAIZA CESAR SILVIO</t>
         </is>
       </c>
       <c r="K68" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>MIERCOLES</t>
+          <t>SABADO</t>
         </is>
       </c>
       <c r="M68" s="2" t="n">
         <v>226</v>
       </c>
     </row>
-    <row r="69" ht="45" customHeight="1">
-      <c r="A69" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="B69" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>11:30 - 12:00</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>Sala 2</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>JAIME FELIPE MEDINA SOTOMAYOR</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>MARCO GALARZA CASTILLO</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="n"/>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>Modelo predictivo del rendimiento deportivo en el fútbol ecuatoriano a  partir del presupuesto institucional y variables competitivas usando  técnicas de Inteligencia Artificial</t>
-        </is>
-      </c>
-      <c r="J69" s="2" t="inlineStr">
-        <is>
-          <t>CASTRO GARCIA DIEGO FERNANDO / PILA CAIZA CESAR SILVIO</t>
-        </is>
-      </c>
-      <c r="K69" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="L69" s="2" t="inlineStr">
-        <is>
-          <t>SABADO</t>
-        </is>
-      </c>
-      <c r="M69" s="2" t="n">
-        <v>226</v>
-      </c>
-    </row>
+    <row r="69" ht="45" customHeight="1"/>
     <row r="70" ht="45" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21481,7 +21427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="14.1"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -24915,17 +24861,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>11:00 - 11:30</t>
+          <t>11:30 - 12:00</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -24934,7 +24880,7 @@
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
@@ -24954,12 +24900,12 @@
       <c r="J64" s="2" t="n"/>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Detección de noticias falsas mediante técnicas de Inteligencia Artificial aplicadas al Procesamiento de Lenguaje Natural en el contexto periodístico</t>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO</t>
+          <t>ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
     </row>
@@ -24969,17 +24915,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>11:30 - 12:00</t>
+          <t>12:00 - 12:30</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -24988,16 +24934,16 @@
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+          <t>DAVID POZO ESPÍN</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -25008,12 +24954,12 @@
       <c r="J65" s="2" t="n"/>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Sistema inteligente de automatización, predicción y atención asistida para  optimizar la gestión de casos en soporte técnico para la empresa  Hispasat en Ecuador</t>
+          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>ALVEAR LEMA EMILIO JOSE</t>
+          <t>LEON MORILLO JOAQUIN ANDRES</t>
         </is>
       </c>
     </row>
@@ -25023,17 +24969,17 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>12:00 - 12:30</t>
+          <t>12:30 - 13:00</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -25042,7 +24988,7 @@
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
@@ -25051,7 +24997,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
+          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -25062,12 +25008,12 @@
       <c r="J66" s="2" t="n"/>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
+          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>LEON MORILLO JOAQUIN ANDRES</t>
+          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
         </is>
       </c>
     </row>
@@ -25077,17 +25023,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>12:30 - 13:00</t>
+          <t>13:00 - 13:30</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -25096,7 +25042,7 @@
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
@@ -25105,7 +25051,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
+          <t>IVÁN ORTIZ</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -25116,12 +25062,12 @@
       <c r="J67" s="2" t="n"/>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
+          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
+          <t>RON LARCO MAURO DANILO</t>
         </is>
       </c>
     </row>
@@ -25131,17 +25077,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>13:00 - 13:30</t>
+          <t>13:30 - 14:00</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -25150,7 +25096,7 @@
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
@@ -25159,7 +25105,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>IVÁN ORTIZ</t>
+          <t>LUIS FERNANDO AGUAS BUCHELI</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -25170,69 +25116,16 @@
       <c r="J68" s="2" t="n"/>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
+          <t>VeriDoc AI: Diseño de un Sistema Inteligente de Asistencia para la Validación  de Completitud y Consistencia Documental en los Procesos de Venta de  Metrocar S.A</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>RON LARCO MAURO DANILO</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="30" customHeight="1">
-      <c r="A69" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>13:30 - 14:00</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>Sala 1</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>DAVID POZO ESPÍN</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>LUIS FERNANDO AGUAS BUCHELI</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>PATRICIO DAVID PONCE</t>
-        </is>
-      </c>
-      <c r="J69" s="2" t="n"/>
-      <c r="K69" s="2" t="inlineStr">
-        <is>
-          <t>VeriDoc AI: Diseño de un Sistema Inteligente de Asistencia para la Validación  de Completitud y Consistencia Documental en los Procesos de Venta de  Metrocar S.A</t>
-        </is>
-      </c>
-      <c r="L69" s="2" t="inlineStr">
-        <is>
           <t>TOBAR LARGO DIANA CRISTINA / VARGAS RIVERA MAYRA SILVANA / NUÑEZ CALAN DENNIS ANDRE</t>
         </is>
       </c>
     </row>
+    <row r="69" ht="30" customHeight="1"/>
     <row r="70" ht="45" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:L70">
@@ -28542,7 +28435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="14.1"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -28948,17 +28841,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>11:00 - 11:30</t>
+          <t>11:30 - 12:00</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -28967,7 +28860,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -28987,12 +28880,12 @@
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Detección de noticias falsas mediante técnicas de Inteligencia Artificial aplicadas al Procesamiento de Lenguaje Natural en el contexto periodístico</t>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO</t>
+          <t>ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
     </row>
@@ -29002,17 +28895,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>11:30 - 12:00</t>
+          <t>12:00 - 12:30</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -29021,16 +28914,16 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+          <t>DAVID POZO ESPÍN</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -29041,12 +28934,12 @@
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Sistema inteligente de automatización, predicción y atención asistida para  optimizar la gestión de casos en soporte técnico para la empresa  Hispasat en Ecuador</t>
+          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>ALVEAR LEMA EMILIO JOSE</t>
+          <t>LEON MORILLO JOAQUIN ANDRES</t>
         </is>
       </c>
     </row>
@@ -29056,17 +28949,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>12:00 - 12:30</t>
+          <t>12:30 - 13:00</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -29075,7 +28968,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -29084,7 +28977,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
+          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -29095,12 +28988,12 @@
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
+          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>LEON MORILLO JOAQUIN ANDRES</t>
+          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
         </is>
       </c>
     </row>
@@ -29110,17 +29003,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>12:30 - 13:00</t>
+          <t>13:00 - 13:30</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -29129,7 +29022,7 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -29138,7 +29031,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
+          <t>IVÁN ORTIZ</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -29149,12 +29042,12 @@
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
+          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
+          <t>RON LARCO MAURO DANILO</t>
         </is>
       </c>
     </row>
@@ -29164,17 +29057,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>13:00 - 13:30</t>
+          <t>13:30 - 14:00</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -29183,7 +29076,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -29192,7 +29085,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>IVÁN ORTIZ</t>
+          <t>LUIS FERNANDO AGUAS BUCHELI</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -29203,69 +29096,16 @@
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
+          <t>VeriDoc AI: Diseño de un Sistema Inteligente de Asistencia para la Validación  de Completitud y Consistencia Documental en los Procesos de Venta de  Metrocar S.A</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>RON LARCO MAURO DANILO</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>13:30 - 14:00</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Sala 1</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>DAVID POZO ESPÍN</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>LUIS FERNANDO AGUAS BUCHELI</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>PATRICIO DAVID PONCE</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>VeriDoc AI: Diseño de un Sistema Inteligente de Asistencia para la Validación  de Completitud y Consistencia Documental en los Procesos de Venta de  Metrocar S.A</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
           <t>TOBAR LARGO DIANA CRISTINA / VARGAS RIVERA MAYRA SILVANA / NUÑEZ CALAN DENNIS ANDRE</t>
         </is>
       </c>
     </row>
+    <row r="13" ht="45" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -29277,7 +29117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="14.1"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -31585,17 +31425,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>11:00 - 11:30</t>
+          <t>11:30 - 12:00</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -31604,7 +31444,7 @@
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -31624,12 +31464,12 @@
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Detección de noticias falsas mediante técnicas de Inteligencia Artificial aplicadas al Procesamiento de Lenguaje Natural en el contexto periodístico</t>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO</t>
+          <t>ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
     </row>
@@ -31639,17 +31479,17 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>11:30 - 12:00</t>
+          <t>12:00 - 12:30</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -31658,16 +31498,16 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+          <t>DAVID POZO ESPÍN</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -31678,12 +31518,12 @@
       <c r="J44" s="2" t="n"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Sistema inteligente de automatización, predicción y atención asistida para  optimizar la gestión de casos en soporte técnico para la empresa  Hispasat en Ecuador</t>
+          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>ALVEAR LEMA EMILIO JOSE</t>
+          <t>LEON MORILLO JOAQUIN ANDRES</t>
         </is>
       </c>
     </row>
@@ -31693,17 +31533,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>12:00 - 12:30</t>
+          <t>12:30 - 13:00</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -31712,7 +31552,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -31721,7 +31561,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
+          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -31732,12 +31572,12 @@
       <c r="J45" s="2" t="n"/>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
+          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>LEON MORILLO JOAQUIN ANDRES</t>
+          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
         </is>
       </c>
     </row>
@@ -31747,17 +31587,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>12:30 - 13:00</t>
+          <t>13:00 - 13:30</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -31766,7 +31606,7 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
@@ -31775,7 +31615,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
+          <t>IVÁN ORTIZ</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -31786,12 +31626,12 @@
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
+          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
+          <t>RON LARCO MAURO DANILO</t>
         </is>
       </c>
     </row>
@@ -31801,17 +31641,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>13:00 - 13:30</t>
+          <t>13:30 - 14:00</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -31820,7 +31660,7 @@
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
@@ -31829,7 +31669,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>IVÁN ORTIZ</t>
+          <t>LUIS FERNANDO AGUAS BUCHELI</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -31840,69 +31680,16 @@
       <c r="J47" s="2" t="n"/>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
+          <t>VeriDoc AI: Diseño de un Sistema Inteligente de Asistencia para la Validación  de Completitud y Consistencia Documental en los Procesos de Venta de  Metrocar S.A</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>RON LARCO MAURO DANILO</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>13:30 - 14:00</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Sala 1</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>DAVID POZO ESPÍN</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>LUIS FERNANDO AGUAS BUCHELI</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>PATRICIO DAVID PONCE</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="n"/>
-      <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>VeriDoc AI: Diseño de un Sistema Inteligente de Asistencia para la Validación  de Completitud y Consistencia Documental en los Procesos de Venta de  Metrocar S.A</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
           <t>TOBAR LARGO DIANA CRISTINA / VARGAS RIVERA MAYRA SILVANA / NUÑEZ CALAN DENNIS ANDRE</t>
         </is>
       </c>
     </row>
+    <row r="48" ht="30" customHeight="1"/>
     <row r="49" ht="45" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: revert oral defense schedule changes and implement programmatic group-based Written Capstone compliance for Lema and Alvear
</commit_message>
<xml_diff>
--- a/data/presentaciones_crcronograma.xlsx
+++ b/data/presentaciones_crcronograma.xlsx
@@ -10587,361 +10587,359 @@
         <v>1</v>
       </c>
       <c r="G117" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>Detección de noticias falsas mediante técnicas de Inteligencia Artificial aplicadas al Procesamiento de Lenguaje Natural en el contexto periodístico</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>SABADO</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="n">
+        <v>226</v>
+      </c>
+      <c r="K117" s="2" t="inlineStr">
+        <is>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+        </is>
+      </c>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+        </is>
+      </c>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO</t>
+        </is>
+      </c>
+      <c r="N117" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="P117" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="Q117" s="2" t="inlineStr">
+        <is>
+          <t>11:00 - 11:30</t>
+        </is>
+      </c>
+      <c r="R117" s="2" t="inlineStr">
+        <is>
+          <t>Sala 1</t>
+        </is>
+      </c>
+      <c r="S117" s="2" t="inlineStr">
+        <is>
+          <t>PATRICIO DAVID PONCE</t>
+        </is>
+      </c>
+      <c r="T117" s="2" t="n"/>
+    </row>
+    <row r="118" ht="60" customHeight="1">
+      <c r="A118" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B118" s="2" t="n">
+        <v>1718453259</v>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>A00026452</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>TALLANA FARINANGO LUIS GUILLERMO</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>luis.tallana@udla.edu.ec</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G118" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>MIERCOLES</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="n">
+        <v>223</v>
+      </c>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>DAVID POZO ESPÍN</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>LEONARDO ARÉVALO RIVERA</t>
+        </is>
+      </c>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
+        </is>
+      </c>
+      <c r="N118" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="P118" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="Q118" s="2" t="inlineStr">
+        <is>
+          <t>11:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="R118" s="2" t="inlineStr">
+        <is>
+          <t>Sala 2</t>
+        </is>
+      </c>
+      <c r="S118" s="2" t="inlineStr">
+        <is>
+          <t>MARCO GALARZA CASTILLO</t>
+        </is>
+      </c>
+      <c r="T118" s="2" t="n"/>
+    </row>
+    <row r="119" ht="45" customHeight="1">
+      <c r="A119" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B119" s="2" t="n">
+        <v>1714286448</v>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>A00875711</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>MENESES SAENZ HOMERO FRANCISCO</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>homero.meneses.saenz@udla.edu.ec</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G119" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>MIERCOLES</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="n">
+        <v>223</v>
+      </c>
+      <c r="K119" s="2" t="inlineStr">
+        <is>
+          <t>DAVID POZO ESPÍN</t>
+        </is>
+      </c>
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t>LEONARDO ARÉVALO RIVERA</t>
+        </is>
+      </c>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
+        </is>
+      </c>
+      <c r="N119" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O119" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="P119" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="Q119" s="2" t="inlineStr">
+        <is>
+          <t>11:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="R119" s="2" t="inlineStr">
+        <is>
+          <t>Sala 2</t>
+        </is>
+      </c>
+      <c r="S119" s="2" t="inlineStr">
+        <is>
+          <t>MARCO GALARZA CASTILLO</t>
+        </is>
+      </c>
+      <c r="T119" s="2" t="n"/>
+    </row>
+    <row r="120" ht="45" customHeight="1">
+      <c r="A120" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B120" s="2" t="n">
+        <v>1721548756</v>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>A00135371</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>QUELAL CRUZ JONATHAN DAVID</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>jonathan.quelal@udla.edu.ec</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G120" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>MIERCOLES</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="n">
+        <v>223</v>
+      </c>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>DAVID POZO ESPÍN</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>LEONARDO ARÉVALO RIVERA</t>
+        </is>
+      </c>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
+        </is>
+      </c>
+      <c r="N120" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O120" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="P120" s="2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="Q120" s="2" t="inlineStr">
+        <is>
+          <t>11:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="R120" s="2" t="inlineStr">
+        <is>
+          <t>Sala 2</t>
+        </is>
+      </c>
+      <c r="S120" s="2" t="inlineStr">
+        <is>
+          <t>MARCO GALARZA CASTILLO</t>
+        </is>
+      </c>
+      <c r="T120" s="2" t="n"/>
+    </row>
+    <row r="121" ht="45" customHeight="1">
+      <c r="A121" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B121" s="2" t="n">
+        <v>1716255763</v>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>A00018648</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>ALVEAR LEMA EMILIO JOSE</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>emilio.alvear@udla.edu.ec</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G121" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="H117" s="2" t="inlineStr">
+      <c r="H121" s="2" t="inlineStr">
         <is>
           <t>Sistema inteligente de automatización, predicción y atención asistida para 
 optimizar la gestión de casos en soporte técnico para la empresa 
 Hispasat en Ecuador</t>
         </is>
       </c>
-      <c r="I117" s="2" t="inlineStr">
-        <is>
-          <t>SABADO</t>
-        </is>
-      </c>
-      <c r="J117" s="2" t="n">
-        <v>226</v>
-      </c>
-      <c r="K117" s="2" t="inlineStr">
-        <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
-        </is>
-      </c>
-      <c r="L117" s="2" t="inlineStr">
-        <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
-        </is>
-      </c>
-      <c r="M117" s="2" t="inlineStr">
-        <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
-        </is>
-      </c>
-      <c r="N117" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="O117" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="P117" s="2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="Q117" s="2" t="inlineStr">
-        <is>
-          <t>11:30 - 12:00</t>
-        </is>
-      </c>
-      <c r="R117" s="2" t="inlineStr">
-        <is>
-          <t>Sala 1</t>
-        </is>
-      </c>
-      <c r="S117" s="2" t="inlineStr">
-        <is>
-          <t>PATRICIO DAVID PONCE</t>
-        </is>
-      </c>
-      <c r="T117" s="2" t="n"/>
-    </row>
-    <row r="118" ht="60" customHeight="1">
-      <c r="A118" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B118" s="2" t="n">
-        <v>1718453259</v>
-      </c>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>A00026452</t>
-        </is>
-      </c>
-      <c r="D118" s="2" t="inlineStr">
-        <is>
-          <t>TALLANA FARINANGO LUIS GUILLERMO</t>
-        </is>
-      </c>
-      <c r="E118" s="2" t="inlineStr">
-        <is>
-          <t>luis.tallana@udla.edu.ec</t>
-        </is>
-      </c>
-      <c r="F118" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G118" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="H118" s="2" t="inlineStr">
-        <is>
-          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
-        </is>
-      </c>
-      <c r="I118" s="2" t="inlineStr">
-        <is>
-          <t>MIERCOLES</t>
-        </is>
-      </c>
-      <c r="J118" s="2" t="n">
-        <v>223</v>
-      </c>
-      <c r="K118" s="2" t="inlineStr">
-        <is>
-          <t>DAVID POZO ESPÍN</t>
-        </is>
-      </c>
-      <c r="L118" s="2" t="inlineStr">
-        <is>
-          <t>LEONARDO ARÉVALO RIVERA</t>
-        </is>
-      </c>
-      <c r="M118" s="2" t="inlineStr">
-        <is>
-          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
-        </is>
-      </c>
-      <c r="N118" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O118" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="P118" s="2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="Q118" s="2" t="inlineStr">
-        <is>
-          <t>11:30 - 12:00</t>
-        </is>
-      </c>
-      <c r="R118" s="2" t="inlineStr">
-        <is>
-          <t>Sala 2</t>
-        </is>
-      </c>
-      <c r="S118" s="2" t="inlineStr">
-        <is>
-          <t>MARCO GALARZA CASTILLO</t>
-        </is>
-      </c>
-      <c r="T118" s="2" t="n"/>
-    </row>
-    <row r="119" ht="45" customHeight="1">
-      <c r="A119" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B119" s="2" t="n">
-        <v>1714286448</v>
-      </c>
-      <c r="C119" s="2" t="inlineStr">
-        <is>
-          <t>A00875711</t>
-        </is>
-      </c>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>MENESES SAENZ HOMERO FRANCISCO</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
-          <t>homero.meneses.saenz@udla.edu.ec</t>
-        </is>
-      </c>
-      <c r="F119" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G119" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="H119" s="2" t="inlineStr">
-        <is>
-          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
-        </is>
-      </c>
-      <c r="I119" s="2" t="inlineStr">
-        <is>
-          <t>MIERCOLES</t>
-        </is>
-      </c>
-      <c r="J119" s="2" t="n">
-        <v>223</v>
-      </c>
-      <c r="K119" s="2" t="inlineStr">
-        <is>
-          <t>DAVID POZO ESPÍN</t>
-        </is>
-      </c>
-      <c r="L119" s="2" t="inlineStr">
-        <is>
-          <t>LEONARDO ARÉVALO RIVERA</t>
-        </is>
-      </c>
-      <c r="M119" s="2" t="inlineStr">
-        <is>
-          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
-        </is>
-      </c>
-      <c r="N119" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O119" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="P119" s="2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="Q119" s="2" t="inlineStr">
-        <is>
-          <t>11:30 - 12:00</t>
-        </is>
-      </c>
-      <c r="R119" s="2" t="inlineStr">
-        <is>
-          <t>Sala 2</t>
-        </is>
-      </c>
-      <c r="S119" s="2" t="inlineStr">
-        <is>
-          <t>MARCO GALARZA CASTILLO</t>
-        </is>
-      </c>
-      <c r="T119" s="2" t="n"/>
-    </row>
-    <row r="120" ht="45" customHeight="1">
-      <c r="A120" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B120" s="2" t="n">
-        <v>1721548756</v>
-      </c>
-      <c r="C120" s="2" t="inlineStr">
-        <is>
-          <t>A00135371</t>
-        </is>
-      </c>
-      <c r="D120" s="2" t="inlineStr">
-        <is>
-          <t>QUELAL CRUZ JONATHAN DAVID</t>
-        </is>
-      </c>
-      <c r="E120" s="2" t="inlineStr">
-        <is>
-          <t>jonathan.quelal@udla.edu.ec</t>
-        </is>
-      </c>
-      <c r="F120" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G120" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="H120" s="2" t="inlineStr">
-        <is>
-          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
-        </is>
-      </c>
-      <c r="I120" s="2" t="inlineStr">
-        <is>
-          <t>MIERCOLES</t>
-        </is>
-      </c>
-      <c r="J120" s="2" t="n">
-        <v>223</v>
-      </c>
-      <c r="K120" s="2" t="inlineStr">
-        <is>
-          <t>DAVID POZO ESPÍN</t>
-        </is>
-      </c>
-      <c r="L120" s="2" t="inlineStr">
-        <is>
-          <t>LEONARDO ARÉVALO RIVERA</t>
-        </is>
-      </c>
-      <c r="M120" s="2" t="inlineStr">
-        <is>
-          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
-        </is>
-      </c>
-      <c r="N120" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O120" s="2" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="P120" s="2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="Q120" s="2" t="inlineStr">
-        <is>
-          <t>11:30 - 12:00</t>
-        </is>
-      </c>
-      <c r="R120" s="2" t="inlineStr">
-        <is>
-          <t>Sala 2</t>
-        </is>
-      </c>
-      <c r="S120" s="2" t="inlineStr">
-        <is>
-          <t>MARCO GALARZA CASTILLO</t>
-        </is>
-      </c>
-      <c r="T120" s="2" t="n"/>
-    </row>
-    <row r="121" ht="45" customHeight="1">
-      <c r="A121" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B121" s="2" t="n">
-        <v>1716255763</v>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>A00018648</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>ALVEAR LEMA EMILIO JOSE</t>
-        </is>
-      </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>emilio.alvear@udla.edu.ec</t>
-        </is>
-      </c>
-      <c r="F121" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G121" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="H121" s="2" t="inlineStr">
-        <is>
-          <t>Sistema inteligente de automatización, predicción y atención asistida para 
-optimizar la gestión de casos en soporte técnico para la empresa 
-Hispasat en Ecuador</t>
-        </is>
-      </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
           <t>SABADO</t>
@@ -10962,7 +10960,7 @@
       </c>
       <c r="M121" s="2" t="inlineStr">
         <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
+          <t>ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
       <c r="N121" s="2" t="n">
@@ -17637,7 +17635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="14.1"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="2"/>
@@ -20923,65 +20921,65 @@
     </row>
     <row r="60" ht="45" customHeight="1">
       <c r="A60" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B60" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>11:30 - 12:00</t>
+          <t>11:00 - 11:30</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Sala 2</t>
+          <t>Sala 1</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>DAVID POZO ESPÍN</t>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>LEONARDO ARÉVALO RIVERA</t>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>MARCO GALARZA CASTILLO</t>
+          <t>PATRICIO DAVID PONCE</t>
         </is>
       </c>
       <c r="H60" s="2" t="n"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
+          <t>Detección de noticias falsas mediante técnicas de Inteligencia Artificial aplicadas al Procesamiento de Lenguaje Natural en el contexto periodístico</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO</t>
         </is>
       </c>
       <c r="K60" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>MIERCOLES</t>
+          <t>SABADO</t>
         </is>
       </c>
       <c r="M60" s="2" t="n">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="61" ht="45" customHeight="1">
       <c r="A61" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B61" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
@@ -20990,60 +20988,62 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Sala 1</t>
+          <t>Sala 2</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+          <t>DAVID POZO ESPÍN</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+          <t>LEONARDO ARÉVALO RIVERA</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>PATRICIO DAVID PONCE</t>
+          <t>MARCO GALARZA CASTILLO</t>
         </is>
       </c>
       <c r="H61" s="2" t="n"/>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
-        </is>
-      </c>
-      <c r="J61" s="2" t="n">
-        <v>2</v>
+          <t>Análisis de equidad y sesgo en el desempeño académico mediante modelos de aprendizaje automático y métricas de justicia algorítmica en el Instituto Tecnológico Pichincha.</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>TALLANA FARINANGO LUIS GUILLERMO / MENESES SAENZ HOMERO FRANCISCO / QUELAL CRUZ JONATHAN DAVID</t>
+        </is>
       </c>
       <c r="K61" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>SABADO</t>
+          <t>MIERCOLES</t>
         </is>
       </c>
       <c r="M61" s="2" t="n">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="62" ht="45" customHeight="1">
       <c r="A62" s="2" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B62" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>08:30 - 09:00</t>
+          <t>11:30 - 12:00</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Sala 2</t>
+          <t>Sala 1</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -21053,23 +21053,23 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>JUAN CARLOS FIGUEROA</t>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>MARCO GALARZA CASTILLO</t>
+          <t>PATRICIO DAVID PONCE</t>
         </is>
       </c>
       <c r="H62" s="2" t="n"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Sistema inteligente de captación, clasificación y predicción de oportunidades de venta mediante un agente de IA en WhatsApp para Clearminds Consultores.</t>
+          <t>Sistema inteligente de automatización, predicción y atención asistida para  optimizar la gestión de casos en soporte técnico para la empresa  Hispasat en Ecuador</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>VILLEGAS ALLAUCA ANTONIO DE JESUS</t>
+          <t>ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
       <c r="K62" s="2" t="n">
@@ -21077,7 +21077,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>MIERCOLES</t>
+          <t>SABADO</t>
         </is>
       </c>
       <c r="M62" s="2" t="n">
@@ -21086,124 +21086,124 @@
     </row>
     <row r="63" ht="45" customHeight="1">
       <c r="A63" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B63" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>09:30 - 10:00</t>
+          <t>08:30 - 09:00</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Sala 1</t>
+          <t>Sala 2</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>ANDREA GALLEGOS ANDRADE</t>
+          <t>JUAN CARLOS FIGUEROA</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>PATRICIO DAVID PONCE</t>
+          <t>MARCO GALARZA CASTILLO</t>
         </is>
       </c>
       <c r="H63" s="2" t="n"/>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Análisis de sentimientos y clasificación de negocio para comentarios de encuestas de satisfacción de clientes.</t>
+          <t>Sistema inteligente de captación, clasificación y predicción de oportunidades de venta mediante un agente de IA en WhatsApp para Clearminds Consultores.</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>BEDON CAMPAÑA ADRIAN RUBEN / BEDON RODRIGUEZ JAIRO FABRISIO</t>
+          <t>VILLEGAS ALLAUCA ANTONIO DE JESUS</t>
         </is>
       </c>
       <c r="K63" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>MARTES</t>
+          <t>MIERCOLES</t>
         </is>
       </c>
       <c r="M63" s="2" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="64" ht="45" customHeight="1">
       <c r="A64" s="2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>08:30 - 09:00</t>
+          <t>09:30 - 10:00</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Sala 2</t>
+          <t>Sala 1</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>LUIS CRIOLLO</t>
+          <t>ANDREA GALLEGOS ANDRADE</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>MARCO GALARZA CASTILLO</t>
+          <t>PATRICIO DAVID PONCE</t>
         </is>
       </c>
       <c r="H64" s="2" t="n"/>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Predicción del riesgo de daño a uno mismo y a otros en consultantes que buscan  atención psicológica en un centro de formación en psicoterapia mediante  aprendizaje de máquina a partir de datos clínicos y sociodemográficos</t>
+          <t>Análisis de sentimientos y clasificación de negocio para comentarios de encuestas de satisfacción de clientes.</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>VALDIVIEZO OÑA JORGE ANDRES</t>
+          <t>BEDON CAMPAÑA ADRIAN RUBEN / BEDON RODRIGUEZ JAIRO FABRISIO</t>
         </is>
       </c>
       <c r="K64" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>SABADO</t>
+          <t>MARTES</t>
         </is>
       </c>
       <c r="M64" s="2" t="n">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="2" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>09:30 - 10:00</t>
+          <t>08:30 - 09:00</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -21218,7 +21218,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>PABLO MONCAYO</t>
+          <t>LUIS CRIOLLO</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -21229,12 +21229,12 @@
       <c r="H65" s="2" t="n"/>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Implementación de IA Generativa para los flujos de mercado entre  compañías para Nestlé S.A.</t>
+          <t>Predicción del riesgo de daño a uno mismo y a otros en consultantes que buscan  atención psicológica en un centro de formación en psicoterapia mediante  aprendizaje de máquina a partir de datos clínicos y sociodemográficos</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>POLO EGAS TAMIA EMILIA</t>
+          <t>VALDIVIEZO OÑA JORGE ANDRES</t>
         </is>
       </c>
       <c r="K65" s="2" t="n">
@@ -21242,7 +21242,7 @@
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>MIERCOLES</t>
+          <t>SABADO</t>
         </is>
       </c>
       <c r="M65" s="2" t="n">
@@ -21251,124 +21251,124 @@
     </row>
     <row r="66" ht="60" customHeight="1">
       <c r="A66" s="2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>12:00 - 12:30</t>
+          <t>09:30 - 10:00</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Sala 1</t>
+          <t>Sala 2</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>SANTIAGO SOLÓRZANO LESCANO</t>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>MATEO FERNANDO CÓRDOVA PROAÑO</t>
+          <t>PABLO MONCAYO</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>PATRICIO DAVID PONCE</t>
+          <t>MARCO GALARZA CASTILLO</t>
         </is>
       </c>
       <c r="H66" s="2" t="n"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Implementación de un Proceso de Atención Digital mediante un Chatbot  con Inteligencia Artificial para la Mejora de la Atención al Usuario</t>
+          <t>Implementación de IA Generativa para los flujos de mercado entre  compañías para Nestlé S.A.</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>ESPINOZA AGUILAR CAMILA ALEJANDRA / CUMBAL CUMBAL JOSE ALEXANDER</t>
+          <t>POLO EGAS TAMIA EMILIA</t>
         </is>
       </c>
       <c r="K66" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>MARTES</t>
+          <t>MIERCOLES</t>
         </is>
       </c>
       <c r="M66" s="2" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B67" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>09:30 - 10:00</t>
+          <t>12:00 - 12:30</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Sala 2</t>
+          <t>Sala 1</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>IVÁN ORTIZ</t>
+          <t>MATEO FERNANDO CÓRDOVA PROAÑO</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>MARCO GALARZA CASTILLO</t>
+          <t>PATRICIO DAVID PONCE</t>
         </is>
       </c>
       <c r="H67" s="2" t="n"/>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo de un agente inteligente basado en modelos de lenguaje de gran  escala para la automatización del análisis y respuesta a incidentes de  ciberseguridad</t>
+          <t>Implementación de un Proceso de Atención Digital mediante un Chatbot  con Inteligencia Artificial para la Mejora de la Atención al Usuario</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>BUITRON GONZAGA CRISTHIAN ANDRES</t>
+          <t>ESPINOZA AGUILAR CAMILA ALEJANDRA / CUMBAL CUMBAL JOSE ALEXANDER</t>
         </is>
       </c>
       <c r="K67" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>MIERCOLES</t>
+          <t>MARTES</t>
         </is>
       </c>
       <c r="M67" s="2" t="n">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="68" ht="45" customHeight="1">
       <c r="A68" s="2" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B68" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>11:30 - 12:00</t>
+          <t>09:30 - 10:00</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -21383,7 +21383,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>JAIME FELIPE MEDINA SOTOMAYOR</t>
+          <t>IVÁN ORTIZ</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -21394,27 +21394,81 @@
       <c r="H68" s="2" t="n"/>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Modelo predictivo del rendimiento deportivo en el fútbol ecuatoriano a  partir del presupuesto institucional y variables competitivas usando  técnicas de Inteligencia Artificial</t>
+          <t>Desarrollo de un agente inteligente basado en modelos de lenguaje de gran  escala para la automatización del análisis y respuesta a incidentes de  ciberseguridad</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>CASTRO GARCIA DIEGO FERNANDO / PILA CAIZA CESAR SILVIO</t>
+          <t>BUITRON GONZAGA CRISTHIAN ANDRES</t>
         </is>
       </c>
       <c r="K68" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>SABADO</t>
+          <t>MIERCOLES</t>
         </is>
       </c>
       <c r="M68" s="2" t="n">
         <v>226</v>
       </c>
     </row>
-    <row r="69" ht="45" customHeight="1"/>
+    <row r="69" ht="45" customHeight="1">
+      <c r="A69" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>11:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Sala 2</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>JAIME FELIPE MEDINA SOTOMAYOR</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>MARCO GALARZA CASTILLO</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="n"/>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Modelo predictivo del rendimiento deportivo en el fútbol ecuatoriano a  partir del presupuesto institucional y variables competitivas usando  técnicas de Inteligencia Artificial</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>CASTRO GARCIA DIEGO FERNANDO / PILA CAIZA CESAR SILVIO</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>SABADO</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="n">
+        <v>226</v>
+      </c>
+    </row>
     <row r="70" ht="45" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21427,7 +21481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="14.1"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -24861,17 +24915,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
           <t>11:30</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>11:30 - 12:00</t>
+          <t>11:00 - 11:30</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -24880,7 +24934,7 @@
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
@@ -24900,12 +24954,12 @@
       <c r="J64" s="2" t="n"/>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
+          <t>Detección de noticias falsas mediante técnicas de Inteligencia Artificial aplicadas al Procesamiento de Lenguaje Natural en el contexto periodístico</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>ALVEAR LEMA EMILIO JOSE</t>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO</t>
         </is>
       </c>
     </row>
@@ -24915,17 +24969,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>12:00 - 12:30</t>
+          <t>11:30 - 12:00</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -24934,16 +24988,16 @@
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>DAVID POZO ESPÍN</t>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -24954,12 +25008,12 @@
       <c r="J65" s="2" t="n"/>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
+          <t>Sistema inteligente de automatización, predicción y atención asistida para  optimizar la gestión de casos en soporte técnico para la empresa  Hispasat en Ecuador</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>LEON MORILLO JOAQUIN ANDRES</t>
+          <t>ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
     </row>
@@ -24969,17 +25023,17 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>12:30 - 13:00</t>
+          <t>12:00 - 12:30</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -24988,7 +25042,7 @@
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
@@ -24997,7 +25051,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
+          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -25008,12 +25062,12 @@
       <c r="J66" s="2" t="n"/>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
+          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
+          <t>LEON MORILLO JOAQUIN ANDRES</t>
         </is>
       </c>
     </row>
@@ -25023,17 +25077,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
           <t>13:00</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>13:00 - 13:30</t>
+          <t>12:30 - 13:00</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -25042,7 +25096,7 @@
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
@@ -25051,7 +25105,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>IVÁN ORTIZ</t>
+          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -25062,12 +25116,12 @@
       <c r="J67" s="2" t="n"/>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
+          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>RON LARCO MAURO DANILO</t>
+          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
         </is>
       </c>
     </row>
@@ -25077,17 +25131,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>13:30 - 14:00</t>
+          <t>13:00 - 13:30</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -25096,7 +25150,7 @@
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
@@ -25105,7 +25159,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO AGUAS BUCHELI</t>
+          <t>IVÁN ORTIZ</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -25116,16 +25170,69 @@
       <c r="J68" s="2" t="n"/>
       <c r="K68" s="2" t="inlineStr">
         <is>
+          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>RON LARCO MAURO DANILO</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="A69" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>13:30 - 14:00</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Sala 1</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>DAVID POZO ESPÍN</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO AGUAS BUCHELI</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>PATRICIO DAVID PONCE</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="n"/>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
           <t>VeriDoc AI: Diseño de un Sistema Inteligente de Asistencia para la Validación  de Completitud y Consistencia Documental en los Procesos de Venta de  Metrocar S.A</t>
         </is>
       </c>
-      <c r="L68" s="2" t="inlineStr">
+      <c r="L69" s="2" t="inlineStr">
         <is>
           <t>TOBAR LARGO DIANA CRISTINA / VARGAS RIVERA MAYRA SILVANA / NUÑEZ CALAN DENNIS ANDRE</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="30" customHeight="1"/>
     <row r="70" ht="45" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:L70">
@@ -28435,7 +28542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="14.1"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -28841,17 +28948,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>11:30</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>11:30 - 12:00</t>
+          <t>11:00 - 11:30</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -28860,7 +28967,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -28880,12 +28987,12 @@
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
+          <t>Detección de noticias falsas mediante técnicas de Inteligencia Artificial aplicadas al Procesamiento de Lenguaje Natural en el contexto periodístico</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>ALVEAR LEMA EMILIO JOSE</t>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO</t>
         </is>
       </c>
     </row>
@@ -28895,17 +29002,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>12:00 - 12:30</t>
+          <t>11:30 - 12:00</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -28914,16 +29021,16 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>DAVID POZO ESPÍN</t>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -28934,12 +29041,12 @@
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
+          <t>Sistema inteligente de automatización, predicción y atención asistida para  optimizar la gestión de casos en soporte técnico para la empresa  Hispasat en Ecuador</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>LEON MORILLO JOAQUIN ANDRES</t>
+          <t>ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
     </row>
@@ -28949,17 +29056,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>12:30 - 13:00</t>
+          <t>12:00 - 12:30</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -28968,7 +29075,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -28977,7 +29084,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
+          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -28988,12 +29095,12 @@
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
+          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
+          <t>LEON MORILLO JOAQUIN ANDRES</t>
         </is>
       </c>
     </row>
@@ -29003,17 +29110,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>13:00</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>13:00 - 13:30</t>
+          <t>12:30 - 13:00</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -29022,7 +29129,7 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -29031,7 +29138,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>IVÁN ORTIZ</t>
+          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -29042,12 +29149,12 @@
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
+          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>RON LARCO MAURO DANILO</t>
+          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
         </is>
       </c>
     </row>
@@ -29057,17 +29164,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>13:30 - 14:00</t>
+          <t>13:00 - 13:30</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -29076,7 +29183,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -29085,7 +29192,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO AGUAS BUCHELI</t>
+          <t>IVÁN ORTIZ</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -29096,16 +29203,69 @@
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
+          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>RON LARCO MAURO DANILO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>13:30 - 14:00</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Sala 1</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>DAVID POZO ESPÍN</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO AGUAS BUCHELI</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>PATRICIO DAVID PONCE</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
           <t>VeriDoc AI: Diseño de un Sistema Inteligente de Asistencia para la Validación  de Completitud y Consistencia Documental en los Procesos de Venta de  Metrocar S.A</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>TOBAR LARGO DIANA CRISTINA / VARGAS RIVERA MAYRA SILVANA / NUÑEZ CALAN DENNIS ANDRE</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -29117,7 +29277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="14.1"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -31425,17 +31585,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
           <t>11:30</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>11:30 - 12:00</t>
+          <t>11:00 - 11:30</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -31444,7 +31604,7 @@
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -31464,12 +31624,12 @@
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>LEMA CHILIQUINGA PAUL ALEJANDRO / ALVEAR LEMA EMILIO JOSE</t>
+          <t>Detección de noticias falsas mediante técnicas de Inteligencia Artificial aplicadas al Procesamiento de Lenguaje Natural en el contexto periodístico</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>ALVEAR LEMA EMILIO JOSE</t>
+          <t>LEMA CHILIQUINGA PAUL ALEJANDRO</t>
         </is>
       </c>
     </row>
@@ -31479,17 +31639,17 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>12:00 - 12:30</t>
+          <t>11:30 - 12:00</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -31498,16 +31658,16 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>DAVID POZO ESPÍN</t>
+          <t>WILLIAM VILLEGAS CHILIQUINGA</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
+          <t>SANTIAGO SOLÓRZANO LESCANO</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -31518,12 +31678,12 @@
       <c r="J44" s="2" t="n"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
+          <t>Sistema inteligente de automatización, predicción y atención asistida para  optimizar la gestión de casos en soporte técnico para la empresa  Hispasat en Ecuador</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>LEON MORILLO JOAQUIN ANDRES</t>
+          <t>ALVEAR LEMA EMILIO JOSE</t>
         </is>
       </c>
     </row>
@@ -31533,17 +31693,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>12:30 - 13:00</t>
+          <t>12:00 - 12:30</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -31552,7 +31712,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -31561,7 +31721,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
+          <t>CÉSAR ALBERTO LARREA ARAUJO</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -31572,12 +31732,12 @@
       <c r="J45" s="2" t="n"/>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
+          <t>Implementación de un chatbot con procesamiento de lenguaje natural para optimizar la atención a estudiantes interesados en programas de intercambio en la UDLA</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
+          <t>LEON MORILLO JOAQUIN ANDRES</t>
         </is>
       </c>
     </row>
@@ -31587,17 +31747,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
           <t>13:00</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>13:00 - 13:30</t>
+          <t>12:30 - 13:00</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -31606,7 +31766,7 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
@@ -31615,7 +31775,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>IVÁN ORTIZ</t>
+          <t>DIEGO CAMILO MIÑO BRAZZERO</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -31626,12 +31786,12 @@
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
+          <t>(Modelo de automatización y precalificación para la suscripción de líneas de crédito  para empresas B2B ecuatorianas mediante el uso de parámetros cuantitativos de la  empresa Coface Ecuador.)</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>RON LARCO MAURO DANILO</t>
+          <t>TAPIA MENDIETA KATHERINE CRISTINA / SALA CARLOSAMA LEONEL ANDRES / JARA VERA CARLOS ANDRES</t>
         </is>
       </c>
     </row>
@@ -31641,17 +31801,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>13:30 - 14:00</t>
+          <t>13:00 - 13:30</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -31660,7 +31820,7 @@
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
@@ -31669,7 +31829,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO AGUAS BUCHELI</t>
+          <t>IVÁN ORTIZ</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -31680,16 +31840,69 @@
       <c r="J47" s="2" t="n"/>
       <c r="K47" s="2" t="inlineStr">
         <is>
+          <t>MODELO DE DETECCIÓN DE ANOMALÍAS EN LA RED WAN DE EP PETROECUADOR</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>RON LARCO MAURO DANILO</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>13:30 - 14:00</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Sala 1</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>DAVID POZO ESPÍN</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO AGUAS BUCHELI</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>PATRICIO DAVID PONCE</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="n"/>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
           <t>VeriDoc AI: Diseño de un Sistema Inteligente de Asistencia para la Validación  de Completitud y Consistencia Documental en los Procesos de Venta de  Metrocar S.A</t>
         </is>
       </c>
-      <c r="L47" s="2" t="inlineStr">
+      <c r="L48" s="2" t="inlineStr">
         <is>
           <t>TOBAR LARGO DIANA CRISTINA / VARGAS RIVERA MAYRA SILVANA / NUÑEZ CALAN DENNIS ANDRE</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="30" customHeight="1"/>
     <row r="49" ht="45" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>